<commit_message>
Added New Java Code
</commit_message>
<xml_diff>
--- a/M_File_Write_XLSX.xlsx
+++ b/M_File_Write_XLSX.xlsx
@@ -12,48 +12,33 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
-    <t>My</t>
+    <t>sanjeVV</t>
   </si>
   <si>
-    <t>name</t>
+    <t>13-08-2024</t>
   </si>
   <si>
-    <t>is</t>
+    <t>thAKU12</t>
   </si>
   <si>
-    <t>Sanjeev</t>
+    <t>sanRTas</t>
   </si>
   <si>
-    <t>i</t>
+    <t>23-04-2026</t>
   </si>
   <si>
-    <t>am</t>
+    <t>##hAKU1@@</t>
   </si>
   <si>
-    <t>from</t>
+    <t>SERTYanje67</t>
   </si>
   <si>
-    <t>bihar</t>
+    <t>01-09-2026</t>
   </si>
   <si>
-    <t>I</t>
-  </si>
-  <si>
-    <t>have</t>
-  </si>
-  <si>
-    <t>sarted</t>
-  </si>
-  <si>
-    <t>the</t>
-  </si>
-  <si>
-    <t>study</t>
-  </si>
-  <si>
-    <t>31/05/2026</t>
+    <t>hAKU1*&amp;*</t>
   </si>
 </sst>
 </file>
@@ -98,7 +83,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -111,42 +96,27 @@
       <c r="C1" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="D1" t="s" s="0">
-        <v>3</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s" s="0">
         <v>4</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="C2" t="s" s="0">
         <v>5</v>
-      </c>
-      <c r="C2" t="s" s="0">
-        <v>6</v>
-      </c>
-      <c r="D2" t="s" s="0">
-        <v>7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="D3" t="s" s="0">
-        <v>11</v>
-      </c>
-      <c r="E3" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="F3" t="s" s="0">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>